<commit_message>
Jul 17, 2026, 4:04 PM
</commit_message>
<xml_diff>
--- a/clean_oxide_data.xlsx
+++ b/clean_oxide_data.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D237"/>
+  <dimension ref="A1:E237"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -437,6 +437,11 @@
           <t>DeltaG (kJ/mol)</t>
         </is>
       </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Phase</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -455,6 +460,7 @@
       <c r="D2" t="n">
         <v>-0.004184</v>
       </c>
+      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -473,6 +479,11 @@
       <c r="D3" t="n">
         <v>-920.48</v>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -491,6 +502,7 @@
       <c r="D4" t="n">
         <v>-542.0163499665551</v>
       </c>
+      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -509,6 +521,7 @@
       <c r="D5" t="n">
         <v>-648.8908227424757</v>
       </c>
+      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -527,6 +540,11 @@
       <c r="D6" t="n">
         <v>-617.5584</v>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -545,6 +563,11 @@
       <c r="D7" t="n">
         <v>-537.644</v>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -563,6 +586,11 @@
       <c r="D8" t="n">
         <v>-330.536</v>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -581,6 +609,11 @@
       <c r="D9" t="n">
         <v>-322.168</v>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -599,6 +632,11 @@
       <c r="D10" t="n">
         <v>-297.064</v>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -617,6 +655,7 @@
       <c r="D11" t="n">
         <v>-66.944</v>
       </c>
+      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -635,6 +674,11 @@
       <c r="D12" t="n">
         <v>-717.556</v>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -653,6 +697,11 @@
       <c r="D13" t="n">
         <v>-468.608</v>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -671,6 +720,11 @@
       <c r="D14" t="n">
         <v>-928.8480000000001</v>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -689,6 +743,11 @@
       <c r="D15" t="n">
         <v>-765.672</v>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -707,6 +766,11 @@
       <c r="D16" t="n">
         <v>-665.256</v>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -725,6 +789,7 @@
       <c r="D17" t="n">
         <v>-548.104</v>
       </c>
+      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -743,6 +808,11 @@
       <c r="D18" t="n">
         <v>-887.008</v>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -761,6 +831,11 @@
       <c r="D19" t="n">
         <v>-669.4400000000001</v>
       </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -779,6 +854,11 @@
       <c r="D20" t="n">
         <v>-34.65308342857141</v>
       </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -797,6 +877,7 @@
       <c r="D21" t="n">
         <v>-59.6103469496021</v>
       </c>
+      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -815,6 +896,7 @@
       <c r="D22" t="n">
         <v>-139.3272</v>
       </c>
+      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -833,6 +915,7 @@
       <c r="D23" t="n">
         <v>-819.6456000000001</v>
       </c>
+      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -851,6 +934,7 @@
       <c r="D24" t="n">
         <v>-401.2456</v>
       </c>
+      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -869,6 +953,7 @@
       <c r="D25" t="n">
         <v>19.66480000000008</v>
       </c>
+      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -887,6 +972,11 @@
       <c r="D26" t="n">
         <v>-1041.816</v>
       </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -905,6 +995,11 @@
       <c r="D27" t="n">
         <v>-907.928</v>
       </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -923,6 +1018,11 @@
       <c r="D28" t="n">
         <v>-489.528</v>
       </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -941,6 +1041,11 @@
       <c r="D29" t="n">
         <v>-401.664</v>
       </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -959,6 +1064,11 @@
       <c r="D30" t="n">
         <v>-309.616</v>
       </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -977,6 +1087,7 @@
       <c r="D31" t="n">
         <v>-0.004184</v>
       </c>
+      <c r="E31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -995,6 +1106,11 @@
       <c r="D32" t="n">
         <v>-991.6080000000001</v>
       </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1013,6 +1129,7 @@
       <c r="D33" t="n">
         <v>-457.7296000000001</v>
       </c>
+      <c r="E33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1031,6 +1148,11 @@
       <c r="D34" t="n">
         <v>-173.636</v>
       </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1049,6 +1171,11 @@
       <c r="D35" t="n">
         <v>-112.968</v>
       </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1067,6 +1194,7 @@
       <c r="D36" t="n">
         <v>-50.208</v>
       </c>
+      <c r="E36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1085,6 +1213,11 @@
       <c r="D37" t="n">
         <v>171.3709485294115</v>
       </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1103,6 +1236,11 @@
       <c r="D38" t="n">
         <v>-376.56</v>
       </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1121,6 +1259,11 @@
       <c r="D39" t="n">
         <v>-324.26</v>
       </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1139,6 +1282,11 @@
       <c r="D40" t="n">
         <v>-315.892</v>
       </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1157,6 +1305,11 @@
       <c r="D41" t="n">
         <v>-523</v>
       </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1175,6 +1328,11 @@
       <c r="D42" t="n">
         <v>-351.456</v>
       </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1193,6 +1351,11 @@
       <c r="D43" t="n">
         <v>-305.432</v>
       </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1211,6 +1374,11 @@
       <c r="D44" t="n">
         <v>-301.248</v>
       </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1229,6 +1397,11 @@
       <c r="D45" t="n">
         <v>-138.072</v>
       </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1247,6 +1420,11 @@
       <c r="D46" t="n">
         <v>-117.152</v>
       </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -1265,6 +1443,11 @@
       <c r="D47" t="n">
         <v>16.07187301587301</v>
       </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -1283,6 +1466,11 @@
       <c r="D48" t="n">
         <v>29.84530373360244</v>
       </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -1301,6 +1489,7 @@
       <c r="D49" t="n">
         <v>-39.748</v>
       </c>
+      <c r="E49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -1319,6 +1508,11 @@
       <c r="D50" t="n">
         <v>-922.572</v>
       </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -1337,6 +1531,11 @@
       <c r="D51" t="n">
         <v>-733.6051266666653</v>
       </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -1355,6 +1554,11 @@
       <c r="D52" t="n">
         <v>-703.5894095238106</v>
       </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -1373,6 +1577,11 @@
       <c r="D53" t="n">
         <v>-925.0824</v>
       </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -1391,6 +1600,11 @@
       <c r="D54" t="n">
         <v>-764.5119949923322</v>
       </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -1409,6 +1623,11 @@
       <c r="D55" t="n">
         <v>-665.1744598990429</v>
       </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -1427,6 +1646,11 @@
       <c r="D56" t="n">
         <v>-1025.08</v>
       </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -1445,6 +1669,11 @@
       <c r="D57" t="n">
         <v>-873.2008</v>
       </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -1463,6 +1692,11 @@
       <c r="D58" t="n">
         <v>-1025.08</v>
       </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -1481,6 +1715,11 @@
       <c r="D59" t="n">
         <v>-901.3487559633035</v>
       </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -1499,6 +1738,11 @@
       <c r="D60" t="n">
         <v>-733.1174091743126</v>
       </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -1517,6 +1761,11 @@
       <c r="D61" t="n">
         <v>-901.3487559633035</v>
       </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -1535,6 +1784,11 @@
       <c r="D62" t="n">
         <v>-570.7390561467902</v>
       </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -1553,6 +1807,7 @@
       <c r="D63" t="n">
         <v>-414.216</v>
       </c>
+      <c r="E63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -1571,6 +1826,11 @@
       <c r="D64" t="n">
         <v>-214.0630615809841</v>
       </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -1589,6 +1849,11 @@
       <c r="D65" t="n">
         <v>-313.8</v>
       </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -1607,6 +1872,11 @@
       <c r="D66" t="n">
         <v>-300.8296</v>
       </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -1625,6 +1895,7 @@
       <c r="D67" t="n">
         <v>12.13359999999992</v>
       </c>
+      <c r="E67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -1643,6 +1914,7 @@
       <c r="D68" t="n">
         <v>-284.0936</v>
       </c>
+      <c r="E68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -1661,6 +1933,11 @@
       <c r="D69" t="n">
         <v>-661.072</v>
       </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -1679,6 +1956,11 @@
       <c r="D70" t="n">
         <v>-267.776</v>
       </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -1697,6 +1979,11 @@
       <c r="D71" t="n">
         <v>-209.2</v>
       </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -1715,6 +2002,11 @@
       <c r="D72" t="n">
         <v>-919.2248</v>
       </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -1733,6 +2025,11 @@
       <c r="D73" t="n">
         <v>-709.2151234916566</v>
       </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -1751,6 +2048,11 @@
       <c r="D74" t="n">
         <v>-555.6397653401782</v>
       </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -1769,6 +2071,11 @@
       <c r="D75" t="n">
         <v>-305.432</v>
       </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -1787,6 +2094,11 @@
       <c r="D76" t="n">
         <v>-282.0016000000001</v>
       </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -1805,6 +2117,11 @@
       <c r="D77" t="n">
         <v>-267.776</v>
       </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -1823,6 +2140,7 @@
       <c r="D78" t="n">
         <v>-356.8952</v>
       </c>
+      <c r="E78" t="inlineStr"/>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -1841,6 +2159,7 @@
       <c r="D79" t="n">
         <v>-79.49600000000001</v>
       </c>
+      <c r="E79" t="inlineStr"/>
     </row>
     <row r="80">
       <c r="A80" t="inlineStr">
@@ -1859,6 +2178,7 @@
       <c r="D80" t="n">
         <v>-112.5496</v>
       </c>
+      <c r="E80" t="inlineStr"/>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
@@ -1877,6 +2197,11 @@
       <c r="D81" t="n">
         <v>-635.9680000000001</v>
       </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
@@ -1895,6 +2220,11 @@
       <c r="D82" t="n">
         <v>-481.16</v>
       </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
@@ -1913,6 +2243,11 @@
       <c r="D83" t="n">
         <v>-923.8272000000001</v>
       </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
@@ -1931,6 +2266,11 @@
       <c r="D84" t="n">
         <v>-744.9677148788944</v>
       </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -1949,6 +2289,11 @@
       <c r="D85" t="n">
         <v>-687.785175086507</v>
       </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -1967,6 +2312,11 @@
       <c r="D86" t="n">
         <v>-531.3680000000001</v>
       </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -1985,6 +2335,11 @@
       <c r="D87" t="n">
         <v>-172.7992</v>
       </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -2003,6 +2358,11 @@
       <c r="D88" t="n">
         <v>-138.072</v>
       </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -2021,6 +2381,7 @@
       <c r="D89" t="n">
         <v>-0.0004184</v>
       </c>
+      <c r="E89" t="inlineStr"/>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -2039,6 +2400,11 @@
       <c r="D90" t="n">
         <v>-631.784</v>
       </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -2057,6 +2423,11 @@
       <c r="D91" t="n">
         <v>-447.688</v>
       </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -2075,6 +2446,11 @@
       <c r="D92" t="n">
         <v>-435.136</v>
       </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -2093,6 +2469,11 @@
       <c r="D93" t="n">
         <v>-297.064</v>
       </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -2111,6 +2492,7 @@
       <c r="D94" t="n">
         <v>-0.004184</v>
       </c>
+      <c r="E94" t="inlineStr"/>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -2129,6 +2511,11 @@
       <c r="D95" t="n">
         <v>-860.6487999999999</v>
       </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -2147,6 +2534,11 @@
       <c r="D96" t="n">
         <v>-1079.472</v>
       </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -2165,6 +2557,11 @@
       <c r="D97" t="n">
         <v>-723.832</v>
       </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -2183,6 +2580,11 @@
       <c r="D98" t="n">
         <v>-535.552</v>
       </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -2201,6 +2603,11 @@
       <c r="D99" t="n">
         <v>-881.9872</v>
       </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -2219,6 +2626,11 @@
       <c r="D100" t="n">
         <v>-1004.16</v>
       </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -2237,6 +2649,11 @@
       <c r="D101" t="n">
         <v>-895.3760000000001</v>
       </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -2255,6 +2672,11 @@
       <c r="D102" t="n">
         <v>-217.568</v>
       </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -2273,6 +2695,7 @@
       <c r="D103" t="n">
         <v>181.0993513513514</v>
       </c>
+      <c r="E103" t="inlineStr"/>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -2291,6 +2714,11 @@
       <c r="D104" t="n">
         <v>-543.9200000000001</v>
       </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -2309,6 +2737,7 @@
       <c r="D105" t="n">
         <v>-79.49600000000001</v>
       </c>
+      <c r="E105" t="inlineStr"/>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -2327,6 +2756,11 @@
       <c r="D106" t="n">
         <v>-451.872</v>
       </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -2345,6 +2779,11 @@
       <c r="D107" t="n">
         <v>-414.216</v>
       </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -2363,6 +2802,7 @@
       <c r="D108" t="n">
         <v>-374.468</v>
       </c>
+      <c r="E108" t="inlineStr"/>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -2381,6 +2821,11 @@
       <c r="D109" t="n">
         <v>-736.384</v>
       </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -2399,6 +2844,11 @@
       <c r="D110" t="n">
         <v>-510.448</v>
       </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -2417,6 +2867,11 @@
       <c r="D111" t="n">
         <v>-497.896</v>
       </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -2435,6 +2890,11 @@
       <c r="D112" t="n">
         <v>-259.408</v>
       </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -2453,6 +2913,7 @@
       <c r="D113" t="n">
         <v>-0.004184</v>
       </c>
+      <c r="E113" t="inlineStr"/>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -2471,6 +2932,11 @@
       <c r="D114" t="n">
         <v>-468.608</v>
       </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -2489,6 +2955,11 @@
       <c r="D115" t="n">
         <v>-451.872</v>
       </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -2507,6 +2978,11 @@
       <c r="D116" t="n">
         <v>-330.536</v>
       </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -2525,6 +3001,11 @@
       <c r="D117" t="n">
         <v>-322.168</v>
       </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -2543,6 +3024,11 @@
       <c r="D118" t="n">
         <v>-309.1976</v>
       </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -2561,6 +3047,11 @@
       <c r="D119" t="n">
         <v>-957.7176000000001</v>
       </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -2579,6 +3070,11 @@
       <c r="D120" t="n">
         <v>-731.8345048573618</v>
       </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -2597,6 +3093,11 @@
       <c r="D121" t="n">
         <v>-566.6139256746322</v>
       </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -2615,6 +3116,11 @@
       <c r="D122" t="n">
         <v>-186.188</v>
       </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -2633,6 +3139,11 @@
       <c r="D123" t="n">
         <v>-102.508</v>
       </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -2651,6 +3162,7 @@
       <c r="D124" t="n">
         <v>-62.76000000000001</v>
       </c>
+      <c r="E124" t="inlineStr"/>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -2669,6 +3181,7 @@
       <c r="D125" t="n">
         <v>-96.232</v>
       </c>
+      <c r="E125" t="inlineStr"/>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -2687,6 +3200,11 @@
       <c r="D126" t="n">
         <v>-397.48</v>
       </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -2705,6 +3223,11 @@
       <c r="D127" t="n">
         <v>-389.112</v>
       </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -2723,6 +3246,7 @@
       <c r="D128" t="n">
         <v>175.728</v>
       </c>
+      <c r="E128" t="inlineStr"/>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -2741,6 +3265,11 @@
       <c r="D129" t="n">
         <v>-288.696</v>
       </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -2759,6 +3288,11 @@
       <c r="D130" t="n">
         <v>-217.568</v>
       </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -2777,6 +3311,11 @@
       <c r="D131" t="n">
         <v>-121.336</v>
       </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -2795,6 +3334,11 @@
       <c r="D132" t="n">
         <v>-146.44</v>
       </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -2813,6 +3357,7 @@
       <c r="D133" t="n">
         <v>-100.416</v>
       </c>
+      <c r="E133" t="inlineStr"/>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -2831,6 +3376,11 @@
       <c r="D134" t="n">
         <v>-987.8424</v>
       </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -2849,6 +3399,11 @@
       <c r="D135" t="n">
         <v>-757.4508556291377</v>
       </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -2867,6 +3422,11 @@
       <c r="D136" t="n">
         <v>-553.0891251655639</v>
       </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -2885,6 +3445,7 @@
       <c r="D137" t="n">
         <v>-0.004184</v>
       </c>
+      <c r="E137" t="inlineStr"/>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -2903,6 +3464,11 @@
       <c r="D138" t="n">
         <v>-928.8480000000001</v>
       </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -2921,6 +3487,11 @@
       <c r="D139" t="n">
         <v>-774.0400000000001</v>
       </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -2939,6 +3510,7 @@
       <c r="D140" t="n">
         <v>-732.2</v>
       </c>
+      <c r="E140" t="inlineStr"/>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -2957,6 +3529,11 @@
       <c r="D141" t="n">
         <v>-577.3920000000001</v>
       </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -2975,6 +3552,11 @@
       <c r="D142" t="n">
         <v>-401.664</v>
       </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -2993,6 +3575,11 @@
       <c r="D143" t="n">
         <v>-397.48</v>
       </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -3011,6 +3598,7 @@
       <c r="D144" t="n">
         <v>-0.004184</v>
       </c>
+      <c r="E144" t="inlineStr"/>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -3029,6 +3617,7 @@
       <c r="D145" t="n">
         <v>-117.152</v>
       </c>
+      <c r="E145" t="inlineStr"/>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -3047,6 +3636,11 @@
       <c r="D146" t="n">
         <v>-309.616</v>
       </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -3065,6 +3659,11 @@
       <c r="D147" t="n">
         <v>-305.432</v>
       </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -3083,6 +3682,11 @@
       <c r="D148" t="n">
         <v>-188.28</v>
       </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -3101,6 +3705,11 @@
       <c r="D149" t="n">
         <v>-133.888</v>
       </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -3119,6 +3728,7 @@
       <c r="D150" t="n">
         <v>-0.0004184</v>
       </c>
+      <c r="E150" t="inlineStr"/>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -3137,6 +3747,11 @@
       <c r="D151" t="n">
         <v>-920.48</v>
       </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -3155,6 +3770,11 @@
       <c r="D152" t="n">
         <v>-138.072</v>
       </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -3173,6 +3793,11 @@
       <c r="D153" t="n">
         <v>-117.152</v>
       </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -3191,6 +3816,11 @@
       <c r="D154" t="n">
         <v>-112.968</v>
       </c>
+      <c r="E154" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -3209,6 +3839,7 @@
       <c r="D155" t="n">
         <v>-0.004184</v>
       </c>
+      <c r="E155" t="inlineStr"/>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -3227,6 +3858,11 @@
       <c r="D156" t="n">
         <v>-610.0272000000001</v>
       </c>
+      <c r="E156" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
@@ -3245,6 +3881,11 @@
       <c r="D157" t="n">
         <v>-608.3536</v>
       </c>
+      <c r="E157" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
@@ -3263,6 +3904,7 @@
       <c r="D158" t="n">
         <v>-451.0352</v>
       </c>
+      <c r="E158" t="inlineStr"/>
     </row>
     <row r="159">
       <c r="A159" t="inlineStr">
@@ -3281,6 +3923,11 @@
       <c r="D159" t="n">
         <v>-950.1864</v>
       </c>
+      <c r="E159" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="160">
       <c r="A160" t="inlineStr">
@@ -3299,6 +3946,11 @@
       <c r="D160" t="n">
         <v>-810.10919078067</v>
       </c>
+      <c r="E160" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="161">
       <c r="A161" t="inlineStr">
@@ -3317,6 +3969,11 @@
       <c r="D161" t="n">
         <v>-708.1651753159841</v>
       </c>
+      <c r="E161" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="162">
       <c r="A162" t="inlineStr">
@@ -3335,6 +3992,11 @@
       <c r="D162" t="n">
         <v>-476.976</v>
       </c>
+      <c r="E162" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" t="inlineStr">
@@ -3353,6 +4015,11 @@
       <c r="D163" t="n">
         <v>-129.704</v>
       </c>
+      <c r="E163" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="164">
       <c r="A164" t="inlineStr">
@@ -3371,6 +4038,11 @@
       <c r="D164" t="n">
         <v>-974.8720000000001</v>
       </c>
+      <c r="E164" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="165">
       <c r="A165" t="inlineStr">
@@ -3389,6 +4061,11 @@
       <c r="D165" t="n">
         <v>-857.72</v>
       </c>
+      <c r="E165" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="166">
       <c r="A166" t="inlineStr">
@@ -3407,6 +4084,11 @@
       <c r="D166" t="n">
         <v>-485.344</v>
       </c>
+      <c r="E166" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="167">
       <c r="A167" t="inlineStr">
@@ -3425,6 +4107,11 @@
       <c r="D167" t="n">
         <v>-443.504</v>
       </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
@@ -3443,6 +4130,11 @@
       <c r="D168" t="n">
         <v>-280.328</v>
       </c>
+      <c r="E168" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
@@ -3461,6 +4153,11 @@
       <c r="D169" t="n">
         <v>-802.4912</v>
       </c>
+      <c r="E169" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
@@ -3479,6 +4176,11 @@
       <c r="D170" t="n">
         <v>-747.6808</v>
       </c>
+      <c r="E170" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
@@ -3497,6 +4199,11 @@
       <c r="D171" t="n">
         <v>-937.6344</v>
       </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
@@ -3515,6 +4222,11 @@
       <c r="D172" t="n">
         <v>-747.3288126984127</v>
       </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="173">
       <c r="A173" t="inlineStr">
@@ -3533,6 +4245,11 @@
       <c r="D173" t="n">
         <v>-452.8257885225889</v>
       </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
@@ -3551,6 +4268,11 @@
       <c r="D174" t="n">
         <v>-398.9681553113551</v>
       </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="175">
       <c r="A175" t="inlineStr">
@@ -3569,6 +4291,11 @@
       <c r="D175" t="n">
         <v>-597.0202730158737</v>
       </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="176">
       <c r="A176" t="inlineStr">
@@ -3587,6 +4314,11 @@
       <c r="D176" t="n">
         <v>-192.464</v>
       </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
@@ -3605,6 +4337,11 @@
       <c r="D177" t="n">
         <v>-138.072</v>
       </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
@@ -3623,6 +4360,11 @@
       <c r="D178" t="n">
         <v>-8.368</v>
       </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="179">
       <c r="A179" t="inlineStr">
@@ -3641,6 +4383,7 @@
       <c r="D179" t="n">
         <v>-0.004184</v>
       </c>
+      <c r="E179" t="inlineStr"/>
     </row>
     <row r="180">
       <c r="A180" t="inlineStr">
@@ -3659,6 +4402,11 @@
       <c r="D180" t="n">
         <v>-853.5360000000001</v>
       </c>
+      <c r="E180" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="181">
       <c r="A181" t="inlineStr">
@@ -3677,6 +4425,11 @@
       <c r="D181" t="n">
         <v>-569.024</v>
       </c>
+      <c r="E181" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="182">
       <c r="A182" t="inlineStr">
@@ -3695,6 +4448,11 @@
       <c r="D182" t="n">
         <v>-673.624</v>
       </c>
+      <c r="E182" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="183">
       <c r="A183" t="inlineStr">
@@ -3713,6 +4471,7 @@
       <c r="D183" t="n">
         <v>-635.9680000000001</v>
       </c>
+      <c r="E183" t="inlineStr"/>
     </row>
     <row r="184">
       <c r="A184" t="inlineStr">
@@ -3731,6 +4490,7 @@
       <c r="D184" t="n">
         <v>-451.872</v>
       </c>
+      <c r="E184" t="inlineStr"/>
     </row>
     <row r="185">
       <c r="A185" t="inlineStr">
@@ -3749,6 +4509,7 @@
       <c r="D185" t="n">
         <v>-376.56</v>
       </c>
+      <c r="E185" t="inlineStr"/>
     </row>
     <row r="186">
       <c r="A186" t="inlineStr">
@@ -3767,6 +4528,11 @@
       <c r="D186" t="n">
         <v>-665.256</v>
       </c>
+      <c r="E186" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="187">
       <c r="A187" t="inlineStr">
@@ -3785,6 +4551,11 @@
       <c r="D187" t="n">
         <v>-616.5721714285727</v>
       </c>
+      <c r="E187" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -3803,6 +4574,7 @@
       <c r="D188" t="n">
         <v>-419.1190151260513</v>
       </c>
+      <c r="E188" t="inlineStr"/>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
@@ -3821,6 +4593,11 @@
       <c r="D189" t="n">
         <v>-347.786490613267</v>
       </c>
+      <c r="E189" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
@@ -3839,6 +4616,7 @@
       <c r="D190" t="n">
         <v>-607.7507661058419</v>
       </c>
+      <c r="E190" t="inlineStr"/>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
@@ -3857,6 +4635,11 @@
       <c r="D191" t="n">
         <v>-385.6616649859943</v>
       </c>
+      <c r="E191" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="192">
       <c r="A192" t="inlineStr">
@@ -3875,6 +4658,11 @@
       <c r="D192" t="n">
         <v>-318.3941960784311</v>
       </c>
+      <c r="E192" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
@@ -3893,6 +4681,11 @@
       <c r="D193" t="n">
         <v>-605.707914346896</v>
       </c>
+      <c r="E193" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
@@ -3911,6 +4704,11 @@
       <c r="D194" t="n">
         <v>-377.9136470588231</v>
       </c>
+      <c r="E194" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
@@ -3929,6 +4727,7 @@
       <c r="D195" t="n">
         <v>-315.7887893738137</v>
       </c>
+      <c r="E195" t="inlineStr"/>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
@@ -3947,6 +4746,7 @@
       <c r="D196" t="n">
         <v>-280.2605161290326</v>
       </c>
+      <c r="E196" t="inlineStr"/>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
@@ -3965,6 +4765,7 @@
       <c r="D197" t="n">
         <v>-596.22</v>
       </c>
+      <c r="E197" t="inlineStr"/>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
@@ -3983,6 +4784,7 @@
       <c r="D198" t="n">
         <v>-267.776</v>
       </c>
+      <c r="E198" t="inlineStr"/>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
@@ -4001,6 +4803,11 @@
       <c r="D199" t="n">
         <v>-217.568</v>
       </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
@@ -4019,6 +4826,11 @@
       <c r="D200" t="n">
         <v>-55.69723396880405</v>
       </c>
+      <c r="E200" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
@@ -4037,6 +4849,11 @@
       <c r="D201" t="n">
         <v>-213.384</v>
       </c>
+      <c r="E201" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
@@ -4055,6 +4872,7 @@
       <c r="D202" t="n">
         <v>-56.484</v>
       </c>
+      <c r="E202" t="inlineStr"/>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
@@ -4073,6 +4891,11 @@
       <c r="D203" t="n">
         <v>-179.912</v>
       </c>
+      <c r="E203" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
@@ -4091,6 +4914,11 @@
       <c r="D204" t="n">
         <v>-22.5865084745763</v>
       </c>
+      <c r="E204" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="205">
       <c r="A205" t="inlineStr">
@@ -4109,6 +4937,11 @@
       <c r="D205" t="n">
         <v>27.49273758865247</v>
       </c>
+      <c r="E205" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="206">
       <c r="A206" t="inlineStr">
@@ -4127,6 +4960,7 @@
       <c r="D206" t="n">
         <v>78.1840786099293</v>
       </c>
+      <c r="E206" t="inlineStr"/>
     </row>
     <row r="207">
       <c r="A207" t="inlineStr">
@@ -4145,6 +4979,11 @@
       <c r="D207" t="n">
         <v>-125.52</v>
       </c>
+      <c r="E207" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="208">
       <c r="A208" t="inlineStr">
@@ -4163,6 +5002,7 @@
       <c r="D208" t="n">
         <v>62.76000000000001</v>
       </c>
+      <c r="E208" t="inlineStr"/>
     </row>
     <row r="209">
       <c r="A209" t="inlineStr">
@@ -4181,6 +5021,7 @@
       <c r="D209" t="n">
         <v>-0.004184</v>
       </c>
+      <c r="E209" t="inlineStr"/>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
@@ -4199,6 +5040,11 @@
       <c r="D210" t="n">
         <v>-904.1624</v>
       </c>
+      <c r="E210" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -4217,6 +5063,11 @@
       <c r="D211" t="n">
         <v>-839.1127043246134</v>
       </c>
+      <c r="E211" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="212">
       <c r="A212" t="inlineStr">
@@ -4235,6 +5086,11 @@
       <c r="D212" t="n">
         <v>-766.4429014415365</v>
       </c>
+      <c r="E212" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="213">
       <c r="A213" t="inlineStr">
@@ -4253,6 +5109,11 @@
       <c r="D213" t="n">
         <v>-845.168</v>
       </c>
+      <c r="E213" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="214">
       <c r="A214" t="inlineStr">
@@ -4271,6 +5132,11 @@
       <c r="D214" t="n">
         <v>-543.9200000000001</v>
       </c>
+      <c r="E214" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="215">
       <c r="A215" t="inlineStr">
@@ -4289,6 +5155,11 @@
       <c r="D215" t="n">
         <v>-79.85962596259633</v>
       </c>
+      <c r="E215" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="216">
       <c r="A216" t="inlineStr">
@@ -4307,6 +5178,11 @@
       <c r="D216" t="n">
         <v>-139.313554582774</v>
       </c>
+      <c r="E216" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="217">
       <c r="A217" t="inlineStr">
@@ -4325,6 +5201,11 @@
       <c r="D217" t="n">
         <v>-139.313554582774</v>
       </c>
+      <c r="E217" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="218">
       <c r="A218" t="inlineStr">
@@ -4343,6 +5224,11 @@
       <c r="D218" t="n">
         <v>-135.0409038635189</v>
       </c>
+      <c r="E218" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="219">
       <c r="A219" t="inlineStr">
@@ -4361,6 +5247,11 @@
       <c r="D219" t="n">
         <v>-487.436</v>
       </c>
+      <c r="E219" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="220">
       <c r="A220" t="inlineStr">
@@ -4379,6 +5270,7 @@
       <c r="D220" t="n">
         <v>-402.0824</v>
       </c>
+      <c r="E220" t="inlineStr"/>
     </row>
     <row r="221">
       <c r="A221" t="inlineStr">
@@ -4397,6 +5289,11 @@
       <c r="D221" t="n">
         <v>-421.015</v>
       </c>
+      <c r="E221" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -4415,6 +5312,11 @@
       <c r="D222" t="n">
         <v>-433.044</v>
       </c>
+      <c r="E222" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -4433,6 +5335,7 @@
       <c r="D223" t="n">
         <v>-397.48</v>
       </c>
+      <c r="E223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -4451,6 +5354,11 @@
       <c r="D224" t="n">
         <v>-280.328</v>
       </c>
+      <c r="E224" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="225">
       <c r="A225" t="inlineStr">
@@ -4469,6 +5377,11 @@
       <c r="D225" t="n">
         <v>-238.488</v>
       </c>
+      <c r="E225" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="226">
       <c r="A226" t="inlineStr">
@@ -4487,6 +5400,7 @@
       <c r="D226" t="n">
         <v>-217.568</v>
       </c>
+      <c r="E226" t="inlineStr"/>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -4505,6 +5419,11 @@
       <c r="D227" t="n">
         <v>-927.1744</v>
       </c>
+      <c r="E227" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="228">
       <c r="A228" t="inlineStr">
@@ -4523,6 +5442,11 @@
       <c r="D228" t="n">
         <v>-750.3656022096733</v>
       </c>
+      <c r="E228" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="229">
       <c r="A229" t="inlineStr">
@@ -4541,6 +5465,11 @@
       <c r="D229" t="n">
         <v>-576.2328294669865</v>
       </c>
+      <c r="E229" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="230">
       <c r="A230" t="inlineStr">
@@ -4559,6 +5488,11 @@
       <c r="D230" t="n">
         <v>-1001.2312</v>
       </c>
+      <c r="E230" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="231">
       <c r="A231" t="inlineStr">
@@ -4577,6 +5511,11 @@
       <c r="D231" t="n">
         <v>-931.992674566999</v>
       </c>
+      <c r="E231" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="232">
       <c r="A232" t="inlineStr">
@@ -4595,6 +5534,11 @@
       <c r="D232" t="n">
         <v>-560.6560000000001</v>
       </c>
+      <c r="E232" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="233">
       <c r="A233" t="inlineStr">
@@ -4613,6 +5557,11 @@
       <c r="D233" t="n">
         <v>-456.056</v>
       </c>
+      <c r="E233" t="inlineStr">
+        <is>
+          <t>b</t>
+        </is>
+      </c>
     </row>
     <row r="234">
       <c r="A234" t="inlineStr">
@@ -4631,6 +5580,11 @@
       <c r="D234" t="n">
         <v>-37.656</v>
       </c>
+      <c r="E234" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
     </row>
     <row r="235">
       <c r="A235" t="inlineStr">
@@ -4649,6 +5603,7 @@
       <c r="D235" t="n">
         <v>-0.004184</v>
       </c>
+      <c r="E235" t="inlineStr"/>
     </row>
     <row r="236">
       <c r="A236" t="inlineStr">
@@ -4667,6 +5622,11 @@
       <c r="D236" t="n">
         <v>-694.544</v>
       </c>
+      <c r="E236" t="inlineStr">
+        <is>
+          <t>m</t>
+        </is>
+      </c>
     </row>
     <row r="237">
       <c r="A237" t="inlineStr">
@@ -4684,6 +5644,11 @@
       </c>
       <c r="D237" t="n">
         <v>-543.9200000000001</v>
+      </c>
+      <c r="E237" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>